<commit_message>
Add F1, MCC metric
</commit_message>
<xml_diff>
--- a/paper/Table_1_radMLBench.xlsx
+++ b/paper/Table_1_radMLBench.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="92">
   <si>
     <t>Dataset</t>
   </si>
@@ -37,6 +37,9 @@
     <t>Balance</t>
   </si>
   <si>
+    <t>Source</t>
+  </si>
+  <si>
     <t>Ahn2021</t>
   </si>
   <si>
@@ -206,13 +209,94 @@
   </si>
   <si>
     <t>Histological type</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.ejrad.2019.108642</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41598-018-30273-4</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.48550/arXiv.2107.02314</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.7717/peerj.16230</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1007/s13246-023-01300-0</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.7717/peerj.14127</t>
+  </si>
+  <si>
+    <t>http://doi.org/10.1038/ncomms5006</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1371/journal.pmed.1002711</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1371/journal.pone.0292110</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41416-023-02480-y</t>
+  </si>
+  <si>
+    <t>http://doi.org/10.7937/K9/TCIA.2016.HdHpgJLK</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1371/journal.pone.0232639</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1007/s10278-017-9984-3</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.48550/arXiv.1911.08434</t>
+  </si>
+  <si>
+    <t>http://doi.org/10.1148/radiol.12111607</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.media.2021.102155</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1007/s11547-023-01718-2</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.juro.2012.08.095</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41598-019-50849-y</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1371/journal.pone.0237587</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1148/ryai.220058</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41597-022-01560-7</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41598-020-72475-9</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.48550/arXiv.2108.08618</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.7717/peerj.14559</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1371/journal.pone.0300170</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.7717/peerj.17111</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -227,6 +311,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -261,16 +352,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -563,10 +660,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -588,16 +685,19 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D2">
         <v>114</v>
@@ -611,16 +711,19 @@
       <c r="G2">
         <v>55</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D3">
         <v>168</v>
@@ -634,16 +737,19 @@
       <c r="G3">
         <v>66</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D4">
         <v>577</v>
@@ -657,16 +763,19 @@
       <c r="G4">
         <v>52</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D5">
         <v>119</v>
@@ -680,16 +789,19 @@
       <c r="G5">
         <v>26</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D6">
         <v>261</v>
@@ -703,16 +815,19 @@
       <c r="G6">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="H6" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D7">
         <v>279</v>
@@ -726,16 +841,19 @@
       <c r="G7">
         <v>49</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="H7" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D8">
         <v>137</v>
@@ -749,16 +867,19 @@
       <c r="G8">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="H8" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D9">
         <v>293</v>
@@ -772,16 +893,19 @@
       <c r="G9">
         <v>54</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="H9" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D10">
         <v>207</v>
@@ -795,16 +919,19 @@
       <c r="G10">
         <v>29</v>
       </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="H10" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D11">
         <v>183</v>
@@ -818,16 +945,19 @@
       <c r="G11">
         <v>73</v>
       </c>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="H11" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D12">
         <v>212</v>
@@ -841,16 +971,19 @@
       <c r="G12">
         <v>46</v>
       </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="H12" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D13">
         <v>520</v>
@@ -864,16 +997,19 @@
       <c r="G13">
         <v>54</v>
       </c>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="H13" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D14">
         <v>161</v>
@@ -887,16 +1023,19 @@
       <c r="G14">
         <v>57</v>
       </c>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="H14" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D15">
         <v>273</v>
@@ -910,16 +1049,19 @@
       <c r="G15">
         <v>44</v>
       </c>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="H15" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D16">
         <v>159</v>
@@ -933,16 +1075,19 @@
       <c r="G16">
         <v>64</v>
       </c>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="H16" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D17">
         <v>173</v>
@@ -956,16 +1101,19 @@
       <c r="G17">
         <v>66</v>
       </c>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="H17" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B18" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D18">
         <v>144</v>
@@ -979,16 +1127,19 @@
       <c r="G18">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="H18" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D19">
         <v>969</v>
@@ -1002,16 +1153,19 @@
       <c r="G19">
         <v>66</v>
       </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="H19" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D20">
         <v>128</v>
@@ -1025,16 +1179,19 @@
       <c r="G20">
         <v>37</v>
       </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="H20" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D21">
         <v>773</v>
@@ -1048,16 +1205,19 @@
       <c r="G21">
         <v>77</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="H21" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C22" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D22">
         <v>138</v>
@@ -1071,16 +1231,19 @@
       <c r="G22">
         <v>49</v>
       </c>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="H22" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D23">
         <v>260</v>
@@ -1094,16 +1257,19 @@
       <c r="G23">
         <v>49</v>
       </c>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="H23" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D24">
         <v>418</v>
@@ -1117,16 +1283,19 @@
       <c r="G24">
         <v>89</v>
       </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="H24" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D25">
         <v>187</v>
@@ -1140,16 +1309,19 @@
       <c r="G25">
         <v>42</v>
       </c>
-    </row>
-    <row r="26" spans="1:7">
+      <c r="H25" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C26" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D26">
         <v>150</v>
@@ -1163,16 +1335,19 @@
       <c r="G26">
         <v>31</v>
       </c>
-    </row>
-    <row r="27" spans="1:7">
+      <c r="H26" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D27">
         <v>203</v>
@@ -1186,16 +1361,19 @@
       <c r="G27">
         <v>35</v>
       </c>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="H27" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C28" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D28">
         <v>245</v>
@@ -1209,16 +1387,19 @@
       <c r="G28">
         <v>51</v>
       </c>
-    </row>
-    <row r="29" spans="1:7">
+      <c r="H28" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C29" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D29">
         <v>114</v>
@@ -1232,16 +1413,19 @@
       <c r="G29">
         <v>50</v>
       </c>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="H29" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D30">
         <v>186</v>
@@ -1255,16 +1439,19 @@
       <c r="G30">
         <v>51</v>
       </c>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="H30" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B31" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C31" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D31">
         <v>203</v>
@@ -1278,16 +1465,19 @@
       <c r="G31">
         <v>51</v>
       </c>
-    </row>
-    <row r="32" spans="1:7">
+      <c r="H31" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C32" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D32">
         <v>255</v>
@@ -1301,16 +1491,19 @@
       <c r="G32">
         <v>57</v>
       </c>
-    </row>
-    <row r="33" spans="1:7">
+      <c r="H32" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C33" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D33">
         <v>192</v>
@@ -1324,8 +1517,45 @@
       <c r="G33">
         <v>66</v>
       </c>
+      <c r="H33" s="2" t="s">
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1"/>
+    <hyperlink ref="H3" r:id="rId2"/>
+    <hyperlink ref="H4" r:id="rId3"/>
+    <hyperlink ref="H5" r:id="rId4"/>
+    <hyperlink ref="H6" r:id="rId5"/>
+    <hyperlink ref="H7" r:id="rId6"/>
+    <hyperlink ref="H8" r:id="rId7"/>
+    <hyperlink ref="H9" r:id="rId8"/>
+    <hyperlink ref="H10" r:id="rId9"/>
+    <hyperlink ref="H11" r:id="rId10"/>
+    <hyperlink ref="H12" r:id="rId11"/>
+    <hyperlink ref="H13" r:id="rId12"/>
+    <hyperlink ref="H14" r:id="rId13"/>
+    <hyperlink ref="H15" r:id="rId14"/>
+    <hyperlink ref="H16" r:id="rId15"/>
+    <hyperlink ref="H17" r:id="rId16"/>
+    <hyperlink ref="H18" r:id="rId17"/>
+    <hyperlink ref="H19" r:id="rId18"/>
+    <hyperlink ref="H20" r:id="rId19"/>
+    <hyperlink ref="H21" r:id="rId20"/>
+    <hyperlink ref="H22" r:id="rId21"/>
+    <hyperlink ref="H23" r:id="rId22"/>
+    <hyperlink ref="H24" r:id="rId23"/>
+    <hyperlink ref="H25" r:id="rId24"/>
+    <hyperlink ref="H26" r:id="rId25"/>
+    <hyperlink ref="H27" r:id="rId26"/>
+    <hyperlink ref="H28" r:id="rId27"/>
+    <hyperlink ref="H29" r:id="rId28"/>
+    <hyperlink ref="H30" r:id="rId29"/>
+    <hyperlink ref="H31" r:id="rId30"/>
+    <hyperlink ref="H32" r:id="rId31"/>
+    <hyperlink ref="H33" r:id="rId32"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>